<commit_message>
feat: infer RDFModel inheritance from absence of SeMPyRO_inherits_from
Remove the SeMPyRO_add_rdf_model column from the classes sheet. A class
without a defined inheritance now inherits from RDFModel automatically.

Co-Authored-By: Claude Opus 5 (1M context)
</commit_message>
<xml_diff>
--- a/tests/test_input/multi_metadata.xlsx
+++ b/tests/test_input/multi_metadata.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,11 +560,6 @@
           <t>SeMPyRO_annotations_IRI</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>SeMPyRO_add_rdf_model</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -597,11 +592,6 @@
           <t>http://example.com/ClassA</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -632,11 +622,6 @@
       <c r="F3" t="inlineStr">
         <is>
           <t>http://example.com/ClassB</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(shaclplay): read correctly spelled controlled vocabulary column
Co-Authored-By: Claude Opus 5.5 (1M context)
</commit_message>
<xml_diff>
--- a/tests/test_input/multi_metadata.xlsx
+++ b/tests/test_input/multi_metadata.xlsx
@@ -672,7 +672,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Controlled vocabluary (if applicable)</t>
+          <t>Controlled vocabulary (if applicable)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Controlled vocabluary (if applicable)</t>
+          <t>Controlled vocabulary (if applicable)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">

</xml_diff>